<commit_message>
debug and update code so that it able to run M4 and M5 correctly as oreviously it did not run thru on the back end.
</commit_message>
<xml_diff>
--- a/data/figures/phase1/phase1_metrics.xlsx
+++ b/data/figures/phase1/phase1_metrics.xlsx
@@ -519,58 +519,58 @@
         <v>19</v>
       </c>
       <c r="B2">
-        <v>61.298</v>
+        <v>62.34</v>
       </c>
       <c r="C2">
-        <v>6.497</v>
+        <v>7.068</v>
       </c>
       <c r="D2">
-        <v>121</v>
+        <v>184</v>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>99.997</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>0.016</v>
       </c>
       <c r="G2">
-        <v>121</v>
+        <v>184</v>
       </c>
       <c r="H2">
-        <v>563.492</v>
+        <v>546.295</v>
       </c>
       <c r="I2">
-        <v>151.123</v>
+        <v>144.19</v>
       </c>
       <c r="J2">
-        <v>120</v>
+        <v>183</v>
       </c>
       <c r="K2">
-        <v>2172.783</v>
+        <v>2157.574</v>
       </c>
       <c r="L2">
-        <v>22.531</v>
+        <v>30.883</v>
       </c>
       <c r="M2">
-        <v>120</v>
+        <v>183</v>
       </c>
       <c r="N2">
-        <v>20.917</v>
+        <v>22.607</v>
       </c>
       <c r="O2">
-        <v>3.385</v>
+        <v>4.001</v>
       </c>
       <c r="P2">
-        <v>120</v>
+        <v>183</v>
       </c>
       <c r="Q2">
-        <v>55.433</v>
+        <v>56.262</v>
       </c>
       <c r="R2">
-        <v>3.238</v>
+        <v>3.039</v>
       </c>
       <c r="S2">
-        <v>120</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -578,58 +578,58 @@
         <v>20</v>
       </c>
       <c r="B3">
-        <v>76.899</v>
+        <v>75.845</v>
       </c>
       <c r="C3">
-        <v>12.375</v>
+        <v>11.856</v>
       </c>
       <c r="D3">
-        <v>140</v>
+        <v>269</v>
       </c>
       <c r="E3">
-        <v>99.72499999999999</v>
+        <v>99.53400000000001</v>
       </c>
       <c r="F3">
-        <v>1.047</v>
+        <v>1.639</v>
       </c>
       <c r="G3">
-        <v>140</v>
+        <v>269</v>
       </c>
       <c r="H3">
-        <v>570.643</v>
+        <v>566.16</v>
       </c>
       <c r="I3">
-        <v>241.085</v>
+        <v>261.184</v>
       </c>
       <c r="J3">
-        <v>140</v>
+        <v>263</v>
       </c>
       <c r="K3">
-        <v>2214.214</v>
+        <v>2197.89</v>
       </c>
       <c r="L3">
-        <v>89.203</v>
+        <v>94.905</v>
       </c>
       <c r="M3">
-        <v>140</v>
+        <v>263</v>
       </c>
       <c r="N3">
-        <v>23.071</v>
+        <v>23.259</v>
       </c>
       <c r="O3">
-        <v>4.898</v>
+        <v>5.179</v>
       </c>
       <c r="P3">
-        <v>140</v>
+        <v>263</v>
       </c>
       <c r="Q3">
-        <v>57.164</v>
+        <v>57.129</v>
       </c>
       <c r="R3">
-        <v>3.067</v>
+        <v>3.031</v>
       </c>
       <c r="S3">
-        <v>140</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -637,58 +637,58 @@
         <v>21</v>
       </c>
       <c r="B4">
-        <v>74.40300000000001</v>
+        <v>74.002</v>
       </c>
       <c r="C4">
-        <v>9.526</v>
+        <v>9.888</v>
       </c>
       <c r="D4">
-        <v>60</v>
+        <v>132</v>
       </c>
       <c r="E4">
-        <v>95.762</v>
+        <v>95.562</v>
       </c>
       <c r="F4">
-        <v>4.758</v>
+        <v>4.957</v>
       </c>
       <c r="G4">
-        <v>60</v>
+        <v>132</v>
       </c>
       <c r="H4">
-        <v>839.35</v>
+        <v>811.913</v>
       </c>
       <c r="I4">
-        <v>210.949</v>
+        <v>227.693</v>
       </c>
       <c r="J4">
-        <v>60</v>
+        <v>126</v>
       </c>
       <c r="K4">
-        <v>2034.933</v>
+        <v>2037.159</v>
       </c>
       <c r="L4">
-        <v>194.348</v>
+        <v>203.146</v>
       </c>
       <c r="M4">
-        <v>60</v>
+        <v>126</v>
       </c>
       <c r="N4">
-        <v>32.333</v>
+        <v>32.619</v>
       </c>
       <c r="O4">
-        <v>3.758</v>
+        <v>4.312</v>
       </c>
       <c r="P4">
-        <v>60</v>
+        <v>126</v>
       </c>
       <c r="Q4">
-        <v>58.983</v>
+        <v>58.944</v>
       </c>
       <c r="R4">
-        <v>0.129</v>
+        <v>0.23</v>
       </c>
       <c r="S4">
-        <v>60</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -696,58 +696,58 @@
         <v>22</v>
       </c>
       <c r="B5">
-        <v>79.89</v>
+        <v>80.63200000000001</v>
       </c>
       <c r="C5">
-        <v>4.283</v>
+        <v>3.834</v>
       </c>
       <c r="D5">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="E5">
         <v>99.985</v>
       </c>
       <c r="F5">
-        <v>0.054</v>
+        <v>0.064</v>
       </c>
       <c r="G5">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="H5">
-        <v>180.575</v>
+        <v>182.188</v>
       </c>
       <c r="I5">
-        <v>45.528</v>
+        <v>44.532</v>
       </c>
       <c r="J5">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="K5">
-        <v>2143.5</v>
+        <v>2145.7</v>
       </c>
       <c r="L5">
-        <v>21.848</v>
+        <v>20.256</v>
       </c>
       <c r="M5">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="N5">
-        <v>16.2</v>
+        <v>16.45</v>
       </c>
       <c r="O5">
-        <v>2.267</v>
+        <v>3.101</v>
       </c>
       <c r="P5">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="Q5">
-        <v>56.625</v>
+        <v>56.55</v>
       </c>
       <c r="R5">
-        <v>2.272</v>
+        <v>2.343</v>
       </c>
       <c r="S5">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:19">
@@ -755,58 +755,58 @@
         <v>23</v>
       </c>
       <c r="B6">
-        <v>82.33</v>
+        <v>80.798</v>
       </c>
       <c r="C6">
-        <v>10.338</v>
+        <v>10.275</v>
       </c>
       <c r="D6">
-        <v>80</v>
+        <v>149</v>
       </c>
       <c r="E6">
-        <v>99.518</v>
+        <v>99.158</v>
       </c>
       <c r="F6">
-        <v>1.352</v>
+        <v>2.133</v>
       </c>
       <c r="G6">
-        <v>80</v>
+        <v>149</v>
       </c>
       <c r="H6">
-        <v>705.85</v>
+        <v>717.657</v>
       </c>
       <c r="I6">
-        <v>191.51</v>
+        <v>223.898</v>
       </c>
       <c r="J6">
-        <v>80</v>
+        <v>143</v>
       </c>
       <c r="K6">
-        <v>2255.462</v>
+        <v>2232.923</v>
       </c>
       <c r="L6">
-        <v>99.104</v>
+        <v>117.169</v>
       </c>
       <c r="M6">
-        <v>80</v>
+        <v>143</v>
       </c>
       <c r="N6">
-        <v>26.162</v>
+        <v>26.692</v>
       </c>
       <c r="O6">
-        <v>3.025</v>
+        <v>3.211</v>
       </c>
       <c r="P6">
-        <v>80</v>
+        <v>143</v>
       </c>
       <c r="Q6">
-        <v>58.738</v>
+        <v>58.769</v>
       </c>
       <c r="R6">
-        <v>0.59</v>
+        <v>0.54</v>
       </c>
       <c r="S6">
-        <v>80</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -814,13 +814,13 @@
         <v>24</v>
       </c>
       <c r="B7">
-        <v>82.73999999999999</v>
+        <v>81.908</v>
       </c>
       <c r="C7">
-        <v>2.811</v>
+        <v>3.488</v>
       </c>
       <c r="D7">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E7">
         <v>100</v>
@@ -829,43 +829,43 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H7">
-        <v>190.6</v>
+        <v>182.075</v>
       </c>
       <c r="I7">
-        <v>59.685</v>
+        <v>55.637</v>
       </c>
       <c r="J7">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K7">
-        <v>2161.75</v>
+        <v>2158.625</v>
       </c>
       <c r="L7">
-        <v>17.814</v>
+        <v>15.511</v>
       </c>
       <c r="M7">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="N7">
-        <v>15.25</v>
+        <v>15.15</v>
       </c>
       <c r="O7">
-        <v>2.268</v>
+        <v>2.497</v>
       </c>
       <c r="P7">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="Q7">
-        <v>54.6</v>
+        <v>54.5</v>
       </c>
       <c r="R7">
-        <v>3.676</v>
+        <v>3.83</v>
       </c>
       <c r="S7">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:19">
@@ -873,58 +873,58 @@
         <v>25</v>
       </c>
       <c r="B8">
-        <v>86.372</v>
+        <v>85.822</v>
       </c>
       <c r="C8">
         <v>3.128</v>
       </c>
       <c r="D8">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="E8">
-        <v>99.928</v>
+        <v>99.938</v>
       </c>
       <c r="F8">
-        <v>0.171</v>
+        <v>0.15</v>
       </c>
       <c r="G8">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="H8">
-        <v>606.65</v>
+        <v>570.174</v>
       </c>
       <c r="I8">
-        <v>92.02</v>
+        <v>105.268</v>
       </c>
       <c r="J8">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="K8">
-        <v>2251.35</v>
+        <v>2249.565</v>
       </c>
       <c r="L8">
-        <v>56.418</v>
+        <v>57.97</v>
       </c>
       <c r="M8">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="N8">
-        <v>28.4</v>
+        <v>28.696</v>
       </c>
       <c r="O8">
-        <v>2.371</v>
+        <v>2.897</v>
       </c>
       <c r="P8">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="Q8">
-        <v>58.95</v>
+        <v>58.848</v>
       </c>
       <c r="R8">
-        <v>0.224</v>
+        <v>0.363</v>
       </c>
       <c r="S8">
-        <v>20</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:19">
@@ -932,58 +932,58 @@
         <v>26</v>
       </c>
       <c r="B9">
-        <v>87.807</v>
+        <v>87.19499999999999</v>
       </c>
       <c r="C9">
-        <v>2.322</v>
+        <v>2.761</v>
       </c>
       <c r="D9">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="E9">
-        <v>99.998</v>
+        <v>99.992</v>
       </c>
       <c r="F9">
-        <v>0.011</v>
+        <v>0.045</v>
       </c>
       <c r="G9">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="H9">
-        <v>618.75</v>
+        <v>594.26</v>
       </c>
       <c r="I9">
-        <v>102.007</v>
+        <v>100.646</v>
       </c>
       <c r="J9">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="K9">
-        <v>2301.917</v>
+        <v>2288.19</v>
       </c>
       <c r="L9">
-        <v>24.145</v>
+        <v>48.623</v>
       </c>
       <c r="M9">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="N9">
-        <v>24.933</v>
+        <v>25.58</v>
       </c>
       <c r="O9">
-        <v>2.162</v>
+        <v>2.768</v>
       </c>
       <c r="P9">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="Q9">
-        <v>58.667</v>
+        <v>58.68</v>
       </c>
       <c r="R9">
-        <v>0.655</v>
+        <v>0.618</v>
       </c>
       <c r="S9">
-        <v>60</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>